<commit_message>
feat: homologação SU-024 — 5 geometrias, 10 associações
- GEO-SU-024 (marco superior / correr / veneziana camarão maxim-ar)
- Delta real ~3.2% lido no catálogo impresso; OCR VS (0.959) era erro conhecido
- Pendentes: SU-025, SU-056, SU-280

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curadoria/biblioteca_curadoria.xlsx
+++ b/curadoria/biblioteca_curadoria.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="80">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -117,6 +117,15 @@
     <t xml:space="preserve">Peso 0.908 kg/m (Alcoa) confirmado. Equivalencia visual confirmada. Contorno preciso pendente.</t>
   </si>
   <si>
+    <t xml:space="preserve">GEO-SU-024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marco Superior / Correr / Veneziana camarão para maxim-ar — família Suprema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delta peso ~3.2% conforme peso lido por Bruno no catálogo impresso da Vitral Sul — o OCR havia lido 0.959 (erro conhecido de OCR; Alcoa índice: 1.024). Equivalência visual confirmada. Contorno preciso pendente.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Perfil</t>
   </si>
   <si>
@@ -207,6 +216,18 @@
     <t xml:space="preserve">VitralSul: catálogo pág 74, PDF físico pág 74. Família local: Nobile 2.5.</t>
   </si>
   <si>
+    <t xml:space="preserve">ALCOA-SU-024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcoa: catálogo pág ~160, PDF físico pág ~173.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VITRALSUL-SU-024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VitralSul: catálogo pág ~75. Família local: Nobile 2.5.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Código</t>
   </si>
   <si>
@@ -225,13 +246,10 @@
     <t xml:space="preserve">Proveniência dos pesos</t>
   </si>
   <si>
-    <t xml:space="preserve">SU-024</t>
+    <t xml:space="preserve">SU-025</t>
   </si>
   <si>
     <t xml:space="preserve">Alcoa: índice do catálogo (texto nativo). Vitral Sul: OCR das páginas raster (confiança menor). Medição: 2026-07-09.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SU-025</t>
   </si>
   <si>
     <t xml:space="preserve">SU-056</t>
@@ -663,7 +681,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -854,6 +872,37 @@
         <v>30</v>
       </c>
     </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -870,7 +919,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -885,36 +934,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>13</v>
@@ -923,24 +972,24 @@
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
@@ -949,24 +998,24 @@
         <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>21</v>
@@ -975,24 +1024,24 @@
         <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>21</v>
@@ -1001,24 +1050,24 @@
         <v>18</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
@@ -1027,24 +1076,24 @@
         <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
@@ -1053,24 +1102,24 @@
         <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>27</v>
@@ -1079,24 +1128,24 @@
         <v>18</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>27</v>
@@ -1105,16 +1154,68 @@
         <v>18</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H9" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>60</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1133,7 +1234,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1146,123 +1247,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1.024</v>
+        <v>0.973</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.959</v>
+        <v>0.919</v>
       </c>
       <c r="D2" s="4" t="n">
         <f aca="false">ABS(B2-C2)/MAX(B2,C2)</f>
-        <v>0.0634765625000001</v>
+        <v>0.0554984583761562</v>
       </c>
       <c r="E2" s="2" t="str">
-        <f aca="false">IF(D2&lt;$B$8,"✓ bate","⚠ olhar desenho")</f>
-        <v>⚠ olhar desenho</v>
+        <f aca="false">IF(D2&lt;$B$7,"✓ bate","⚠ olhar desenho")</f>
+        <v>✓ bate</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.973</v>
+        <v>0.539</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.919</v>
+        <v>0.519</v>
       </c>
       <c r="D3" s="4" t="n">
         <f aca="false">ABS(B3-C3)/MAX(B3,C3)</f>
-        <v>0.0554984583761562</v>
+        <v>0.0371057513914657</v>
       </c>
       <c r="E3" s="2" t="str">
-        <f aca="false">IF(D3&lt;$B$8,"✓ bate","⚠ olhar desenho")</f>
+        <f aca="false">IF(D3&lt;$B$7,"✓ bate","⚠ olhar desenho")</f>
         <v>✓ bate</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.539</v>
+        <v>1.006</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.519</v>
+        <v>0.969</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">ABS(B4-C4)/MAX(B4,C4)</f>
-        <v>0.0371057513914657</v>
+        <v>0.036779324055666</v>
       </c>
       <c r="E4" s="2" t="str">
-        <f aca="false">IF(D4&lt;$B$8,"✓ bate","⚠ olhar desenho")</f>
+        <f aca="false">IF(D4&lt;$B$7,"✓ bate","⚠ olhar desenho")</f>
         <v>✓ bate</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>1.006</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.969</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <f aca="false">ABS(B5-C5)/MAX(B5,C5)</f>
-        <v>0.036779324055666</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <f aca="false">IF(D5&lt;$B$8,"✓ bate","⚠ olhar desenho")</f>
-        <v>✓ bate</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="7" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="7" t="n">
         <v>0.06</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>73</v>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: descrição da GEO-SU-024 — remover 'maxim-ar' (engano do operador)
Correção registrada na _nota para preservar a trilha de auditoria.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curadoria/biblioteca_curadoria.xlsx
+++ b/curadoria/biblioteca_curadoria.xlsx
@@ -120,10 +120,10 @@
     <t xml:space="preserve">GEO-SU-024</t>
   </si>
   <si>
-    <t xml:space="preserve">Marco Superior / Correr / Veneziana camarão para maxim-ar — família Suprema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delta peso ~3.2% conforme peso lido por Bruno no catálogo impresso da Vitral Sul — o OCR havia lido 0.959 (erro conhecido de OCR; Alcoa índice: 1.024). Equivalência visual confirmada. Contorno preciso pendente.</t>
+    <t xml:space="preserve">Marco Superior / Correr / Veneziana camarão — família Suprema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delta peso ~3.2% conforme peso lido por Bruno no catálogo impresso da Vitral Sul — o OCR havia lido 0.959 (erro conhecido de OCR; Alcoa índice: 1.024). Equivalência visual confirmada. Contorno preciso pendente. CORRECAO: descricao anterior incluia 'maxim-ar' por engano do operador — removido.</t>
   </si>
   <si>
     <t xml:space="preserve">Perfil</t>

</xml_diff>

<commit_message>
feat: homologação SU-025 — 6 geometrias, 12 associações
- GEO-SU-025 (marco inferior / correr / veneziana camarão), par do SU-024
- Delta peso 5.5%, dentro da tolerância
- Pendentes: SU-056, SU-280

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curadoria/biblioteca_curadoria.xlsx
+++ b/curadoria/biblioteca_curadoria.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="86">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -126,6 +126,15 @@
     <t xml:space="preserve">Delta peso ~3.2% conforme peso lido por Bruno no catálogo impresso da Vitral Sul — o OCR havia lido 0.959 (erro conhecido de OCR; Alcoa índice: 1.024). Equivalência visual confirmada. Contorno preciso pendente. CORRECAO: descricao anterior incluia 'maxim-ar' por engano do operador — removido.</t>
   </si>
   <si>
+    <t xml:space="preserve">GEO-SU-025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marco Inferior / Correr / Veneziana camarão — família Suprema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Par do SU-024 (marco superior). Equivalência visual confirmada. Contorno preciso pendente.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Perfil</t>
   </si>
   <si>
@@ -228,6 +237,18 @@
     <t xml:space="preserve">VitralSul: catálogo pág ~75. Família local: Nobile 2.5.</t>
   </si>
   <si>
+    <t xml:space="preserve">ALCOA-SU-025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcoa: catálogo ~pág 160, PDF físico ~pág 173.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VITRALSUL-SU-025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VitralSul: catálogo ~pág 75. Família local: Nobile 2.5.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Código</t>
   </si>
   <si>
@@ -246,13 +267,10 @@
     <t xml:space="preserve">Proveniência dos pesos</t>
   </si>
   <si>
-    <t xml:space="preserve">SU-025</t>
+    <t xml:space="preserve">SU-056</t>
   </si>
   <si>
     <t xml:space="preserve">Alcoa: índice do catálogo (texto nativo). Vitral Sul: OCR das páginas raster (confiança menor). Medição: 2026-07-09.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SU-056</t>
   </si>
   <si>
     <t xml:space="preserve">SU-280</t>
@@ -681,7 +699,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -903,6 +921,37 @@
         <v>33</v>
       </c>
     </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -919,7 +968,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -934,36 +983,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>13</v>
@@ -972,24 +1021,24 @@
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
@@ -998,24 +1047,24 @@
         <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>21</v>
@@ -1024,24 +1073,24 @@
         <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>21</v>
@@ -1050,24 +1099,24 @@
         <v>18</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
@@ -1076,24 +1125,24 @@
         <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
@@ -1102,24 +1151,24 @@
         <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>27</v>
@@ -1128,24 +1177,24 @@
         <v>18</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>27</v>
@@ -1154,24 +1203,24 @@
         <v>18</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>31</v>
@@ -1180,24 +1229,24 @@
         <v>18</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>31</v>
@@ -1206,16 +1255,68 @@
         <v>18</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1234,7 +1335,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1247,101 +1348,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.973</v>
+        <v>0.539</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.919</v>
+        <v>0.519</v>
       </c>
       <c r="D2" s="4" t="n">
         <f aca="false">ABS(B2-C2)/MAX(B2,C2)</f>
-        <v>0.0554984583761562</v>
+        <v>0.0371057513914657</v>
       </c>
       <c r="E2" s="2" t="str">
-        <f aca="false">IF(D2&lt;$B$7,"✓ bate","⚠ olhar desenho")</f>
+        <f aca="false">IF(D2&lt;$B$6,"✓ bate","⚠ olhar desenho")</f>
         <v>✓ bate</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.539</v>
+        <v>1.006</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.519</v>
+        <v>0.969</v>
       </c>
       <c r="D3" s="4" t="n">
         <f aca="false">ABS(B3-C3)/MAX(B3,C3)</f>
-        <v>0.0371057513914657</v>
+        <v>0.036779324055666</v>
       </c>
       <c r="E3" s="2" t="str">
-        <f aca="false">IF(D3&lt;$B$7,"✓ bate","⚠ olhar desenho")</f>
+        <f aca="false">IF(D3&lt;$B$6,"✓ bate","⚠ olhar desenho")</f>
         <v>✓ bate</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>1.006</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0.969</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <f aca="false">ABS(B4-C4)/MAX(B4,C4)</f>
-        <v>0.036779324055666</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <f aca="false">IF(D4&lt;$B$7,"✓ bate","⚠ olhar desenho")</f>
-        <v>✓ bate</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B7" s="7" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="7" t="n">
         <v>0.06</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>79</v>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: homologação SU-056 — 7 geometrias, 14 associações
- GEO-SU-056 (montante mão de amigo)
- Pendente: SU-280

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curadoria/biblioteca_curadoria.xlsx
+++ b/curadoria/biblioteca_curadoria.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="92">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -135,6 +135,15 @@
     <t xml:space="preserve">Par do SU-024 (marco superior). Equivalência visual confirmada. Contorno preciso pendente.</t>
   </si>
   <si>
+    <t xml:space="preserve">GEO-SU-056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montante mão de amigo — família Suprema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equivalência visual confirmada. Contorno preciso pendente.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Perfil</t>
   </si>
   <si>
@@ -249,6 +258,18 @@
     <t xml:space="preserve">VitralSul: catálogo ~pág 75. Família local: Nobile 2.5.</t>
   </si>
   <si>
+    <t xml:space="preserve">ALCOA-SU-056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcoa: catálogo ~pág 163, PDF físico ~pág 176.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VITRALSUL-SU-056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VitralSul: catálogo ~pág 78. Família local: Nobile 2.5.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Código</t>
   </si>
   <si>
@@ -267,13 +288,10 @@
     <t xml:space="preserve">Proveniência dos pesos</t>
   </si>
   <si>
-    <t xml:space="preserve">SU-056</t>
+    <t xml:space="preserve">SU-280</t>
   </si>
   <si>
     <t xml:space="preserve">Alcoa: índice do catálogo (texto nativo). Vitral Sul: OCR das páginas raster (confiança menor). Medição: 2026-07-09.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SU-280</t>
   </si>
   <si>
     <t xml:space="preserve">Tolerância Δ peso:</t>
@@ -699,7 +717,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -952,6 +970,37 @@
         <v>36</v>
       </c>
     </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -968,7 +1017,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -983,36 +1032,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>13</v>
@@ -1021,24 +1070,24 @@
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
@@ -1047,24 +1096,24 @@
         <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>21</v>
@@ -1073,24 +1122,24 @@
         <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>21</v>
@@ -1099,24 +1148,24 @@
         <v>18</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
@@ -1125,24 +1174,24 @@
         <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
@@ -1151,24 +1200,24 @@
         <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>27</v>
@@ -1177,24 +1226,24 @@
         <v>18</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>27</v>
@@ -1203,24 +1252,24 @@
         <v>18</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>31</v>
@@ -1229,24 +1278,24 @@
         <v>18</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>31</v>
@@ -1255,24 +1304,24 @@
         <v>18</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>34</v>
@@ -1281,24 +1330,24 @@
         <v>18</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>34</v>
@@ -1307,16 +1356,68 @@
         <v>18</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1335,7 +1436,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1348,79 +1449,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.539</v>
+        <v>1.006</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.519</v>
+        <v>0.969</v>
       </c>
       <c r="D2" s="4" t="n">
         <f aca="false">ABS(B2-C2)/MAX(B2,C2)</f>
-        <v>0.0371057513914657</v>
+        <v>0.036779324055666</v>
       </c>
       <c r="E2" s="2" t="str">
-        <f aca="false">IF(D2&lt;$B$6,"✓ bate","⚠ olhar desenho")</f>
+        <f aca="false">IF(D2&lt;$B$5,"✓ bate","⚠ olhar desenho")</f>
         <v>✓ bate</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>1.006</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>0.969</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <f aca="false">ABS(B3-C3)/MAX(B3,C3)</f>
-        <v>0.036779324055666</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <f aca="false">IF(D3&lt;$B$6,"✓ bate","⚠ olhar desenho")</f>
-        <v>✓ bate</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B6" s="7" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="7" t="n">
         <v>0.06</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>85</v>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: homologação SU-280 — lista dos 8 candidatos comuns COMPLETA
- GEO-SU-280 (montante lateral/folha)
- 8 geometrias, 16 associações — todos os códigos comuns Alcoa × Vitral Sul homologados
- Fila de pendentes zerada

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curadoria/biblioteca_curadoria.xlsx
+++ b/curadoria/biblioteca_curadoria.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="96">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -144,6 +144,12 @@
     <t xml:space="preserve">Equivalência visual confirmada. Contorno preciso pendente.</t>
   </si>
   <si>
+    <t xml:space="preserve">GEO-SU-280</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montante lateral/folha — família Suprema</t>
+  </si>
+  <si>
     <t xml:space="preserve">Perfil</t>
   </si>
   <si>
@@ -270,6 +276,18 @@
     <t xml:space="preserve">VitralSul: catálogo ~pág 78. Família local: Nobile 2.5.</t>
   </si>
   <si>
+    <t xml:space="preserve">ALCOA-SU-280</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcoa: catálogo ~pág 165, PDF físico ~pág 178.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VITRALSUL-SU-280</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VitralSul: catálogo ~pág 80. Família local: Nobile 2.5.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Código</t>
   </si>
   <si>
@@ -286,12 +304,6 @@
   </si>
   <si>
     <t xml:space="preserve">Proveniência dos pesos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SU-280</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcoa: índice do catálogo (texto nativo). Vitral Sul: OCR das páginas raster (confiança menor). Medição: 2026-07-09.</t>
   </si>
   <si>
     <t xml:space="preserve">Tolerância Δ peso:</t>
@@ -308,7 +320,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -346,22 +358,15 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="9"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -428,7 +433,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -445,23 +450,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -717,7 +710,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -1001,6 +994,37 @@
         <v>39</v>
       </c>
     </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1017,7 +1041,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -1032,36 +1056,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>13</v>
@@ -1070,24 +1094,24 @@
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
@@ -1096,24 +1120,24 @@
         <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>21</v>
@@ -1122,24 +1146,24 @@
         <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>21</v>
@@ -1148,24 +1172,24 @@
         <v>18</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
@@ -1174,24 +1198,24 @@
         <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
@@ -1200,24 +1224,24 @@
         <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>27</v>
@@ -1226,24 +1250,24 @@
         <v>18</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>27</v>
@@ -1252,24 +1276,24 @@
         <v>18</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>31</v>
@@ -1278,24 +1302,24 @@
         <v>18</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>31</v>
@@ -1304,24 +1328,24 @@
         <v>18</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>34</v>
@@ -1330,24 +1354,24 @@
         <v>18</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>34</v>
@@ -1356,24 +1380,24 @@
         <v>18</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>37</v>
@@ -1382,24 +1406,24 @@
         <v>18</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>37</v>
@@ -1408,16 +1432,68 @@
         <v>18</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>81</v>
+      <c r="C16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1436,7 +1512,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1449,57 +1525,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>1.006</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0.969</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <f aca="false">ABS(B2-C2)/MAX(B2,C2)</f>
-        <v>0.036779324055666</v>
-      </c>
-      <c r="E2" s="2" t="str">
-        <f aca="false">IF(D2&lt;$B$5,"✓ bate","⚠ olhar desenho")</f>
-        <v>✓ bate</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B5" s="7" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="4" t="n">
         <v>0.06</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>91</v>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: expansão para 5 fabricantes — 33 associações em 8 geometrias
- Tamboré (TMS), Centenário (TMS) e ASA (MG25) associados às geometrias existentes
- 6 geometrias agora com 5 fabricantes; SU-280 sem equivalente ASA (registrado)
- ASA-228/230: 1mm de altura, decisão Bruno: mesma GeometriaPadrao
- fix: planilha derivava fabricante como binário Alcoa/VitralSul

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curadoria/biblioteca_curadoria.xlsx
+++ b/curadoria/biblioteca_curadoria.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="135">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -150,6 +150,9 @@
     <t xml:space="preserve">Montante lateral/folha — família Suprema</t>
   </si>
   <si>
+    <t xml:space="preserve">Equivalência visual confirmada. Contorno preciso pendente. ASA (MG25) não possui equivalente catalogado para este perfil.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Perfil</t>
   </si>
   <si>
@@ -286,6 +289,120 @@
   </si>
   <si>
     <t xml:space="preserve">VitralSul: catálogo ~pág 80. Família local: Nobile 2.5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAMBORE-TMS-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamboré</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comparação visual no catálogo impresso — 5 fabricantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamboré TMS-005. Mesma geometria Alcoa/VitralSul já homologada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENTENARIO-TMS-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centenário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centenário TMS-005. Peso difere ligeiramente do Tamboré apesar da mesma nomenclatura — observação de mercado registrada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA-MG25-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA MG25-005. Mesma geometria confirmada por Bruno.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAMBORE-TMS-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamboré TMS-009.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENTENARIO-TMS-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centenário TMS-009. Peso difere ligeiramente do Tamboré.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA-MG25-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA MG25-009.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAMBORE-TMS-056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamboré TMS-056.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENTENARIO-TMS-056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centenário TMS-056. Peso difere ligeiramente do Tamboré.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA-MG25-056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA MG25-056.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAMBORE-TMS-228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamboré TMS-228.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENTENARIO-TMS-228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centenário TMS-228. Peso difere ligeiramente do Tamboré.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA-MG25-228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA MG25-228. Altura 1mm maior que SU-228 — não altera usabilidade. Decisão Bruno: mesma GeometriaPadrao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAMBORE-TMS-230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamboré TMS-230.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENTENARIO-TMS-230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centenário TMS-230. Peso difere ligeiramente do Tamboré.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA-MG25-230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASA MG25-230. Altura 1mm maior que SU-230 — não altera usabilidade. Decisão Bruno: mesma GeometriaPadrao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAMBORE-TMS-280</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamboré TMS-280.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENTENARIO-TMS-280</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centenário TMS-280. Peso difere ligeiramente do Tamboré.</t>
   </si>
   <si>
     <t xml:space="preserve">Código</t>
@@ -1022,7 +1139,7 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1041,7 +1158,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -1056,36 +1173,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>13</v>
@@ -1094,24 +1211,24 @@
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
@@ -1120,24 +1237,24 @@
         <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>21</v>
@@ -1146,24 +1263,24 @@
         <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>21</v>
@@ -1172,24 +1289,24 @@
         <v>18</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
@@ -1198,24 +1315,24 @@
         <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
@@ -1224,24 +1341,24 @@
         <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>27</v>
@@ -1250,24 +1367,24 @@
         <v>18</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>27</v>
@@ -1276,24 +1393,24 @@
         <v>18</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>31</v>
@@ -1302,24 +1419,24 @@
         <v>18</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>31</v>
@@ -1328,24 +1445,24 @@
         <v>18</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>34</v>
@@ -1354,24 +1471,24 @@
         <v>18</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>34</v>
@@ -1380,24 +1497,24 @@
         <v>18</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>37</v>
@@ -1406,24 +1523,24 @@
         <v>18</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>37</v>
@@ -1432,24 +1549,24 @@
         <v>18</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>40</v>
@@ -1458,24 +1575,24 @@
         <v>18</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>40</v>
@@ -1484,16 +1601,458 @@
         <v>18</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1525,27 +2084,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>89</v>
+        <v>128</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>90</v>
+        <v>129</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>91</v>
+        <v>130</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>93</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>94</v>
+        <v>133</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>0.06</v>
@@ -1553,7 +2112,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>95</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>